<commit_message>
Tracker: real state (Tiger Claw), traits.json, dashboard generator
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JjV7LKqjARZJSBEW92E2Pe
</commit_message>
<xml_diff>
--- a/trait-tracker/NFT_Trait_Tracker.xlsx
+++ b/trait-tracker/NFT_Trait_Tracker.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t xml:space="preserve">NFT COLLECTION  ·  ART PROGRESS</t>
   </si>
@@ -76,19 +76,10 @@
     <t xml:space="preserve">Left Arm</t>
   </si>
   <si>
-    <t xml:space="preserve">Gold Watch</t>
+    <t xml:space="preserve">Tiger Claw</t>
   </si>
   <si>
-    <t xml:space="preserve">✓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Right Arm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cigar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiger Claw</t>
+    <t xml:space="preserve">Female versions only (white, tanned, brown)</t>
   </si>
 </sst>
 </file>
@@ -931,25 +922,25 @@
       <c r="A7" s="2"/>
       <c r="B7" s="8" t="n">
         <f aca="false">SUMPRODUCT(($D$11:$O$70="✓")*1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">6*COUNTA($C$11:$C$70)-SUMPRODUCT(($D$11:$O$70="✓")*1)</f>
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">6*COUNTA($C$11:$C$70)</f>
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="11" t="n">
         <f aca="false">IF(COUNTA($C$11:$C$70)=0,0,SUMPRODUCT(($D$11:$O$70="✓")*1)/(6*COUNTA($C$11:$C$70)))</f>
-        <v>0.0555555555555556</v>
+        <v>0</v>
       </c>
       <c r="G7" s="11"/>
       <c r="H7" s="12" t="str">
         <f aca="false">REPT("█",ROUND($F$7*24,0))&amp;REPT("░",24-ROUND($F$7*24,0))</f>
-        <v>█░░░░░░░░░░░░░░░░░░░░░░░</v>
+        <v>░░░░░░░░░░░░░░░░░░░░░░░░</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="12"/>
@@ -1061,9 +1052,7 @@
         <v>18</v>
       </c>
       <c r="D11" s="19"/>
-      <c r="E11" s="20" t="s">
-        <v>19</v>
-      </c>
+      <c r="E11" s="20"/>
       <c r="F11" s="19"/>
       <c r="G11" s="20"/>
       <c r="H11" s="19"/>
@@ -1076,20 +1065,18 @@
       <c r="O11" s="20"/>
       <c r="P11" s="21" t="str">
         <f aca="false">IF($C11="","",SUMPRODUCT(($D11:$O11="✓")*1)&amp;" / 6")</f>
-        <v>1 / 6</v>
-      </c>
-      <c r="Q11" s="22"/>
+        <v>0 / 6</v>
+      </c>
+      <c r="Q11" s="22" t="s">
+        <v>19</v>
+      </c>
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
-      <c r="B12" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="24" t="s">
-        <v>21</v>
-      </c>
+      <c r="B12" s="23"/>
+      <c r="C12" s="24"/>
       <c r="D12" s="25"/>
       <c r="E12" s="26"/>
       <c r="F12" s="25"/>
@@ -1104,7 +1091,7 @@
       <c r="O12" s="26"/>
       <c r="P12" s="27" t="str">
         <f aca="false">IF($C12="","",SUMPRODUCT(($D12:$O12="✓")*1)&amp;" / 6")</f>
-        <v>0 / 6</v>
+        <v/>
       </c>
       <c r="Q12" s="28"/>
       <c r="R12" s="2"/>
@@ -1112,12 +1099,8 @@
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
-      <c r="B13" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>22</v>
-      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="18"/>
       <c r="D13" s="19"/>
       <c r="E13" s="20"/>
       <c r="F13" s="19"/>
@@ -1132,7 +1115,7 @@
       <c r="O13" s="20"/>
       <c r="P13" s="21" t="str">
         <f aca="false">IF($C13="","",SUMPRODUCT(($D13:$O13="✓")*1)&amp;" / 6")</f>
-        <v>0 / 6</v>
+        <v/>
       </c>
       <c r="Q13" s="22"/>
       <c r="R13" s="2"/>

</xml_diff>